<commit_message>
Update monday.com Türkiye research with second-round findings
Sector-by-sector searches, LinkedIn post-link attempts and partner case
study scan added to methodology; notes for Papara and BMS updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TqbqosQvNGMMYWP8i2fjbi
</commit_message>
<xml_diff>
--- a/research/monday-turkiye/monday_turkiye_kullanicilari.xlsx
+++ b/research/monday-turkiye/monday_turkiye_kullanicilari.xlsx
@@ -1936,7 +1936,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Omni Factors'ın LinkedIn şirket sayfasında 'Papara ile çalışmaya başladık… monday.com'un esnek iş süreç yönetimi' duyurusu arama motoru dizininde görünüyor; ancak gönderinin doğrudan açılabilir linki bulunamadı (LinkedIn misafir görünümü yalnızca son ~10 gönderiyi gösteriyor).</t>
+          <t>Omni Factors'ın LinkedIn şirket sayfasında 'Papara ile çalışmaya başladık… monday.com'un esnek iş süreç yönetimi' duyurusu arama motoru dizininde görünüyor; ancak gönderinin doğrudan açılabilir linki bulunamadı. 2. turda tekrar denendi: arama dizini gönderinin varlığını doğruluyor, fakat LinkedIn misafir görünümü (/company/omnifactors ve /posts/) yalnızca son 10 gönderiyi gösteriyor ve gönderi kimliği dizinde yok.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Omni Factors çalışanı Melis Levi'nin LinkedIn paylaşımı (BMS'in Türkiye ofislerinde, Oria Sigorta satın alması sonrası monday.com eğitimi) arama özetinde görünüyor; profil/gönderi misafir erişimine kapalı (HTTP 999).</t>
+          <t>Omni Factors çalışanı Melis Levi'nin LinkedIn paylaşımı (BMS'in Türkiye ofislerinde, Oria Sigorta satın alması sonrası monday.com eğitimi) arama özetinde görünüyor; profil/gönderi misafir erişimine kapalı (HTTP 999). Bağlam doğrulandı: BMS'in Oria Sigorta'yı satın alması 22 Mayıs 2025'te BMS Group'tan Kerim Gürkan'ın LinkedIn paylaşımıyla duyurulmuş; eğitim gönderisinin kendisine ise ulaşılamadı.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2616,7 +2616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -2716,12 +2716,19 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ERİŞİLEMEYEN KAYNAKLAR: Kariyer.net (bot doğrulaması 'Basılı Tutun'), Indeed TR (403), Glassdoor (403), Yenibiris (403), SecretCV (410), Jooble (403), G2 (403), TrustRadius (403), SaaSHub (403), Trustpilot (403), Ekşi Sözlük (403), Wayback Machine ve Common Crawl (bağlantı reddedildi), LinkedIn profilleri ve eski gönderiler (999/giriş), BuiltWith ve PublicWWW tam listeleri (ücretli). LinkedIn iş araması yalnızca AÇIK ilanları ve sorgu başına ~500 sonucu döndürüyor; kapanmış ilanlar görülemedi.</t>
+          <t>2. TUR (kullanıcı isteğiyle): (a) Papara/BMS/Dimes LinkedIn gönderi linkleri için 3 arama + LinkedIn misafir sayfaları (/company/omnifactors, /posts/, tr.linkedin.com, Papara şirket sayfası) denendi → gönderilerin varlığı arama dizininde doğrulandı ama açılabilir link elde edilemedi; (b) 13 sektör için 24 ek Türkçe/İngilizce sorgu (yazılım/SaaS 3, ajans 3, e-ticaret 2, perakende 2, üretim 2, inşaat/gayrimenkul 2, lojistik 2, finans/sigorta 2, sağlık 2, eğitim 2, enerji/telekom 2, kamu/STK 2) → yeni doğrulanabilir şirket yok; çıkan iki ipucu (PSM Awards 2025 proje kataloğu PDF'i, BThaber röportajı) tam metinde monday.com içermiyor; (c) Adaptavist'in 71 benzersiz vaka çalışması (sitemap) tarandı: monday.com vakaları Asepeyo (İspanya), Froghop (İngiltere), Millennia (Hırvatistan) — Türk müşteri yok; Evatro ve Involit WordPress API'lerinde monday.com vaka çalışması yok (Evatro'da yalnızca 'Monday.Com Nedir?' yazısı). EKAP (kamu ihale) kayıtları önerildi ama captcha nedeniyle denenmedi.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>ERİŞİLEMEYEN KAYNAKLAR: Kariyer.net (bot doğrulaması 'Basılı Tutun'), Indeed TR (403), Glassdoor (403), Yenibiris (403), SecretCV (410), Jooble (403), G2 (403), TrustRadius (403), SaaSHub (403), Trustpilot (403), Ekşi Sözlük (403), Wayback Machine ve Common Crawl (bağlantı reddedildi), LinkedIn profilleri ve eski gönderiler (999/giriş), BuiltWith ve PublicWWW tam listeleri (ücretli). LinkedIn iş araması yalnızca AÇIK ilanları ve sorgu başına ~500 sonucu döndürüyor; kapanmış ilanlar görülemedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>LİSTE NEDEN EKSİK OLABİLİR: (1) Türkiye'nin en büyük ilan sitesi Kariyer.net taranamadı; (2) yalnızca şu an açık ilanlar görülebildi; (3) LinkedIn gönderileri/profilleri (en zengin F/B kaynağı) giriş gerektiriyor; (4) monday.com Türkiye'ye özel müşteri hikayesi yayınlamıyor; (5) tek resmi Türk partnerinin referansları logo düzeyinde ve ürün belirtmiyor; (6) sektör bazlı tarama LinkedIn'de sektör yerine rol/şehir üzerinden yapıldı, her sektör için ayrı 3 sorgu yapılmadı. 50+ hedefine kanıtsız isimle ulaşmak yerine liste 24 kayıtta bırakıldı.</t>
         </is>

</xml_diff>